<commit_message>
Fix mis-match: 동국대학교 WISE campus library wrongly assigned to 본교
lib row "동국대학교 WISE캠퍼스 학술정보원" (space-separated, not the
parenthesized "동국대학교(WISE)" form) was matching the bare "동국대학교"
full-name prefix in tier 1 before the WISE keyword check ever ran,
so the row silently landed on the main campus instead of the branch
school. Moved the 5-school main/branch keyword check ahead of the
generic full-name prefix tier. Regenerated both exports; total rows
442 matched libraries + 14 library-less schools = 456 (previously
miscounted as 457 due to this bug).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017djwwG8ViyvYqjXRRMm63e
</commit_message>
<xml_diff>
--- a/data/대학도서관_장애학생지원센터_대상기관목록.xlsx
+++ b/data/대학도서관_장애학생지원센터_대상기관목록.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="대상기관 목록" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="캠퍼스별 상세" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="제외 및 특이사항" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상기관 목록" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="캠퍼스별 상세" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="제외 및 특이사항" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4745,16 +4745,16 @@
         </is>
       </c>
       <c r="G64" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>동국대학교 WISE캠퍼스 학술정보원</t>
+          <t>동국대학교 중앙도서관</t>
         </is>
       </c>
       <c r="I64" s="3" t="inlineStr">
         <is>
-          <t>동국대학교 WISE캠퍼스 학술정보원; 동국대학교 중앙도서관</t>
+          <t>동국대학교 중앙도서관</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
@@ -4776,11 +4776,7 @@
           <t>O</t>
         </is>
       </c>
-      <c r="O64" s="3" t="inlineStr">
-        <is>
-          <t>대학도서관 2개 캠퍼스 통계 존재</t>
-        </is>
-      </c>
+      <c r="O64" s="3" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4814,10 +4810,18 @@
         </is>
       </c>
       <c r="G65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" s="2" t="inlineStr"/>
-      <c r="I65" s="3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>동국대학교 WISE캠퍼스 학술정보원</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>동국대학교 WISE캠퍼스 학술정보원</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
           <t>O</t>
@@ -4839,7 +4843,7 @@
       </c>
       <c r="O65" s="3" t="inlineStr">
         <is>
-          <t>KERIS 도서관 통계 없음 / [교육부고시비고] 경주캠퍼스→WISE캠퍼스('22.4.26)</t>
+          <t>[교육부고시비고] 경주캠퍼스→WISE캠퍼스('22.4.26)</t>
         </is>
       </c>
     </row>
@@ -26640,7 +26644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F139"/>
+  <dimension ref="A1:F137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -27092,7 +27096,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:국립강릉원주대학교</t>
         </is>
       </c>
     </row>
@@ -27124,7 +27128,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:국립강릉원주대학교</t>
         </is>
       </c>
     </row>
@@ -27636,7 +27640,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:서라벌대학교</t>
         </is>
       </c>
     </row>
@@ -28027,86 +28031,86 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>동국대학교</t>
+          <t>명지대학교</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>동국대학교 WISE캠퍼스 학술정보원</t>
+          <t>명지대학교_본교</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 43명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>동국대학교</t>
+          <t>명지대학교</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>동국대학교 중앙도서관</t>
+          <t>명지대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 108명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>명지대학교</t>
+          <t>국립목포대학교</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>명지대학교_본교</t>
+          <t>국립목포대학교 도서관</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -28116,39 +28120,39 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 43명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>명지대학교</t>
+          <t>국립목포대학교</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>명지대학교_제2캠퍼스</t>
+          <t>전남도립대학교 도서관</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 108명, 지원센터유무 O</t>
+          <t>override:전남도립대학교</t>
         </is>
       </c>
     </row>
@@ -28160,27 +28164,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>국립목포대학교 도서관</t>
+          <t>국립목포대학교(담양캠퍼스)_제2캠퍼스</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
         </is>
       </c>
     </row>
@@ -28192,17 +28196,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>전남도립대학교 도서관</t>
+          <t>국립목포대학교_본교</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -28212,61 +28216,61 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>장애재학생(학부) 23명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>국립목포대학교</t>
+          <t>백석대학교</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>국립목포대학교(담양캠퍼스)_제2캠퍼스</t>
+          <t>백석대학교 도서관(서울)</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>국립목포대학교</t>
+          <t>백석대학교</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>국립목포대학교_본교</t>
+          <t>백석대학교 도서관(천안)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -28276,14 +28280,14 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 23명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>백석대학교</t>
+          <t>상명대학교</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -28293,7 +28297,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>백석대학교 도서관(서울)</t>
+          <t>상명대학교 서울캠퍼스 학술정보관</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -28315,7 +28319,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>백석대학교</t>
+          <t>상명대학교</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -28325,7 +28329,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>백석대학교 도서관(천안)</t>
+          <t>상명대학교 천안캠퍼스 학술정보관</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -28335,7 +28339,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -28352,17 +28356,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>상명대학교 서울캠퍼스 학술정보관</t>
+          <t>상명대학교_본교</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -28372,7 +28376,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 22명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -28384,17 +28388,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>상명대학교 천안캠퍼스 학술정보관</t>
+          <t>상명대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -28404,14 +28408,14 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 20명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>상명대학교</t>
+          <t>신한대학교</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -28421,7 +28425,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>상명대학교_본교</t>
+          <t>신한대학교_본교</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -28436,14 +28440,14 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 22명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 1명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>상명대학교</t>
+          <t>신한대학교</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -28453,7 +28457,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>상명대학교_제2캠퍼스</t>
+          <t>신한대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -28468,29 +28472,29 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 20명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 4명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>신한대학교</t>
+          <t>아주대학교</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>신한대학교_본교</t>
+          <t>아주대학교 도서관</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -28500,46 +28504,46 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 1명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>신한대학교</t>
+          <t>아주대학교</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>신한대학교_제2캠퍼스</t>
+          <t>아주대학교 의학문헌정보센터</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 4명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>아주대학교</t>
+          <t>국립경국대학교</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -28549,7 +28553,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>아주대학교 도서관</t>
+          <t>국립경국대학교 예천캠퍼스도서관</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -28571,7 +28575,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>아주대학교</t>
+          <t>국립경국대학교</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -28581,7 +28585,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>아주대학교 의학문헌정보센터</t>
+          <t>국립경국대학교 중앙도서관</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -28603,22 +28607,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>국립경국대학교</t>
+          <t>안양대학교</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>국립경국대학교 예천캠퍼스도서관</t>
+          <t>안양대학교_본교</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -28628,61 +28632,61 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 3명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>국립경국대학교</t>
+          <t>안양대학교</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>국립경국대학교 중앙도서관</t>
+          <t>안양대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>안양대학교</t>
+          <t>연세대학교</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>안양대학교_본교</t>
+          <t>연세대학교 의학도서관</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -28692,46 +28696,46 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 3명, 지원센터유무 O</t>
+          <t>keyword_main</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>안양대학교</t>
+          <t>연세대학교</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>안양대학교_제2캠퍼스</t>
+          <t>연세대학교 학술문화처 도서관</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
+          <t>keyword_main</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>연세대학교</t>
+          <t>연세대학교(미래)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -28741,7 +28745,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>연세대학교 의학도서관</t>
+          <t>연세대학교(미래) 원주캠퍼스 의학도서관</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -28751,19 +28755,19 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>캠퍼스</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>keyword_branch</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>연세대학교</t>
+          <t>연세대학교(미래)</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -28773,7 +28777,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>연세대학교 학술문화처 도서관</t>
+          <t>연세대학교(미래) 학술정보원</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -28783,19 +28787,19 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>캠퍼스</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>keyword_branch</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>연세대학교(미래)</t>
+          <t>영남대학교</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -28805,7 +28809,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>연세대학교(미래) 원주캠퍼스 의학도서관</t>
+          <t>영남대학교 도서관</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -28815,7 +28819,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -28827,7 +28831,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>연세대학교(미래)</t>
+          <t>영남대학교</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -28837,7 +28841,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>연세대학교(미래) 학술정보원</t>
+          <t>영남대학교 의과대학 의학도서관</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -28847,7 +28851,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -28859,54 +28863,54 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>영남대학교</t>
+          <t>영산대학교</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>영남대학교 도서관</t>
+          <t>영산대학교(양산)_제2캠퍼스</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 9명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>영남대학교</t>
+          <t>영산대학교</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>영남대학교 의과대학 의학도서관</t>
+          <t>영산대학교(해운대)_본교</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -28916,14 +28920,14 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 20명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>영산대학교</t>
+          <t>예원예술대학교</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -28933,7 +28937,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>영산대학교(양산)_제2캠퍼스</t>
+          <t>예원예술대학교_본교</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -28943,19 +28947,19 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 9명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>영산대학교</t>
+          <t>예원예술대학교</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -28965,7 +28969,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>영산대학교(해운대)_본교</t>
+          <t>예원예술대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -28975,34 +28979,34 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 20명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>예원예술대학교</t>
+          <t>원광대학교</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>예원예술대학교_본교</t>
+          <t>원광대학교 도서관</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -29012,61 +29016,61 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>예원예술대학교</t>
+          <t>원광대학교</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>예원예술대학교_제2캠퍼스</t>
+          <t>원광보건대학교 도서관</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
+          <t>override:원광보건대학교</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>원광대학교</t>
+          <t>을지대학교</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>원광대학교 도서관</t>
+          <t>을지대학교_본교</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -29076,39 +29080,39 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 0명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>원광대학교</t>
+          <t>을지대학교</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>원광보건대학교 도서관</t>
+          <t>을지대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>장애재학생(학부) 4명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -29125,7 +29129,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>을지대학교_본교</t>
+          <t>을지대학교_제3캠퍼스</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -29135,83 +29139,83 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제3캠퍼스</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 0명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 2명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>을지대학교</t>
+          <t>인제대학교</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>을지대학교_제2캠퍼스</t>
+          <t>인제대학교 백인제기념도서관</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 4명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>을지대학교</t>
+          <t>인제대학교</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>을지대학교_제3캠퍼스</t>
+          <t>인제대학교 의학도서관</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>제3캠퍼스</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 2명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>인제대학교</t>
+          <t>인천가톨릭대학교</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -29221,7 +29225,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>인제대학교 백인제기념도서관</t>
+          <t>인천가톨릭대학교 도서관</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -29243,7 +29247,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>인제대학교</t>
+          <t>인천가톨릭대학교</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -29253,7 +29257,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>인제대학교 의학도서관</t>
+          <t>인천가톨릭대학교 송도국제캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -29280,17 +29284,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교 도서관</t>
+          <t>인천가톨릭대학교_본교</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -29300,7 +29304,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
         </is>
       </c>
     </row>
@@ -29312,17 +29316,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교 송도국제캠퍼스 도서관</t>
+          <t>인천가톨릭대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -29332,14 +29336,14 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교</t>
+          <t>전남대학교</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -29349,7 +29353,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교_본교</t>
+          <t>전남대학교_본교</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -29364,14 +29368,14 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 0명, 지원센터유무 X</t>
+          <t>장애재학생(학부) 86명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교</t>
+          <t>전남대학교</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -29381,7 +29385,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>인천가톨릭대학교_제2캠퍼스</t>
+          <t>전남대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -29396,29 +29400,29 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 6명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 3명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>전남대학교</t>
+          <t>중앙대학교</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>전남대학교_본교</t>
+          <t>중앙대학교 서울캠퍼스 학술정보원</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -29428,29 +29432,29 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 86명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>전남대학교</t>
+          <t>중앙대학교</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>전남대학교_제2캠퍼스</t>
+          <t>중앙대학교 제2캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -29460,7 +29464,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 3명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
@@ -29472,17 +29476,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>중앙대학교 서울캠퍼스 학술정보원</t>
+          <t>중앙대학교_본교</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -29492,7 +29496,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 21명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -29504,17 +29508,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>중앙대학교 제2캠퍼스 도서관</t>
+          <t>중앙대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -29524,29 +29528,29 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 11명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>중앙대학교</t>
+          <t>국립창원대학교</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>중앙대학교_본교</t>
+          <t>경남도립거창대학 도서관</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -29556,39 +29560,39 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 21명, 지원센터유무 O</t>
+          <t>override:경남도립거창대학</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>중앙대학교</t>
+          <t>국립창원대학교</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>중앙대학교_제2캠퍼스</t>
+          <t>경남도립남해대학 도서관</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 11명, 지원센터유무 O</t>
+          <t>override:경남도립남해대학</t>
         </is>
       </c>
     </row>
@@ -29605,7 +29609,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>경남도립거창대학 도서관</t>
+          <t>국립창원대학교 도서관</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -29620,7 +29624,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
@@ -29632,27 +29636,27 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>경남도립남해대학 도서관</t>
+          <t>국립창원대학교(거창캠퍼스)_제2캠퍼스</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>장애재학생(학부) 10명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -29664,27 +29668,27 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>국립창원대학교 도서관</t>
+          <t>국립창원대학교(남해캠퍼스)_제3캠퍼스</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제3캠퍼스</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 12명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -29701,7 +29705,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>국립창원대학교(거창캠퍼스)_제2캠퍼스</t>
+          <t>국립창원대학교_본교</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -29711,66 +29715,66 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 10명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 39명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>국립창원대학교</t>
+          <t>한국외국어대학교</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>국립창원대학교(남해캠퍼스)_제3캠퍼스</t>
+          <t>한국외국어대학교 글로벌캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>제3캠퍼스</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 12명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>국립창원대학교</t>
+          <t>한국외국어대학교</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>국립창원대학교_본교</t>
+          <t>한국외국어대학교 도서관</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -29780,14 +29784,14 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 39명, 지원센터유무 O</t>
+          <t>full_prefix</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>한국외국어대학교</t>
+          <t>한동대학교</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -29797,7 +29801,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>한국외국어대학교 글로벌캠퍼스 도서관</t>
+          <t>한동대학교 국제법률대학원 도서관</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -29807,7 +29811,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -29819,7 +29823,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>한국외국어대학교</t>
+          <t>한동대학교</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -29829,7 +29833,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>한국외국어대학교 도서관</t>
+          <t>한동대학교 학술정보관</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -29851,7 +29855,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>한동대학교</t>
+          <t>한신대학교</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -29861,7 +29865,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>한동대학교 국제법률대학원 도서관</t>
+          <t>한신대학교 신학대학원 장공도서관</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -29883,7 +29887,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>한동대학교</t>
+          <t>한신대학교</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -29893,7 +29897,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>한동대학교 학술정보관</t>
+          <t>한신대학교 중앙도서관</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -29915,7 +29919,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>한신대학교</t>
+          <t>홍익대학교</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -29925,7 +29929,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>한신대학교 신학대학원 장공도서관</t>
+          <t>홍익대학교 문정 도서관</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -29935,7 +29939,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -29947,7 +29951,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>한신대학교</t>
+          <t>홍익대학교</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -29957,7 +29961,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>한신대학교 중앙도서관</t>
+          <t>홍익대학교 중앙도서관</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -29984,27 +29988,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>홍익대학교 문정 도서관</t>
+          <t>홍익대학교_본교</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 8명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
@@ -30016,34 +30020,34 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>대학도서관</t>
+          <t>장애학생지원센터</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>홍익대학교 중앙도서관</t>
+          <t>홍익대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>KERIS</t>
+          <t>장애학생지원센터 현황조사</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>본교</t>
+          <t>제2캠퍼스</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>full_prefix</t>
+          <t>장애재학생(학부) 5명, 지원센터유무 X</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>홍익대학교</t>
+          <t>경인교육대학교</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -30053,7 +30057,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>홍익대학교_본교</t>
+          <t>경인교육대학교_본교</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -30068,14 +30072,14 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 8명, 지원센터유무 O</t>
+          <t>장애재학생(학부) 37명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>홍익대학교</t>
+          <t>경인교육대학교</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -30085,7 +30089,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>홍익대학교_제2캠퍼스</t>
+          <t>경인교육대학교_제2캠퍼스</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -30100,29 +30104,29 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 5명, 지원센터유무 X</t>
+          <t>장애재학생(학부) 31명, 지원센터유무 O</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>경인교육대학교</t>
+          <t>한국폴리텍 I 대학</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>경인교육대학교_본교</t>
+          <t>한국폴리텍Ⅰ대학서울강서캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -30132,39 +30136,39 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 37명, 지원센터유무 O</t>
+          <t>override:한국폴리텍Ⅰ대학</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>경인교육대학교</t>
+          <t>한국폴리텍 I 대학</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>장애학생지원센터</t>
+          <t>대학도서관</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>경인교육대학교_제2캠퍼스</t>
+          <t>한국폴리텍Ⅰ대학서울정수캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>장애학생지원센터 현황조사</t>
+          <t>KERIS</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>제2캠퍼스</t>
+          <t>본교</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>장애재학생(학부) 31명, 지원센터유무 O</t>
+          <t>override:한국폴리텍Ⅰ대학</t>
         </is>
       </c>
     </row>
@@ -30181,7 +30185,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅰ대학서울강서캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅰ대학성남캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -30196,7 +30200,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅰ대학</t>
         </is>
       </c>
     </row>
@@ -30213,7 +30217,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅰ대학서울정수캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅰ대학제주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -30228,14 +30232,14 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅰ대학</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>한국폴리텍 I 대학</t>
+          <t>한국폴리텍 II 대학</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -30245,7 +30249,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅰ대학성남캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅱ대학남인천캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -30260,14 +30264,14 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅱ대학</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>한국폴리텍 I 대학</t>
+          <t>한국폴리텍 II 대학</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -30277,7 +30281,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅰ대학제주캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅱ대학화성캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -30292,14 +30296,14 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅱ대학</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>한국폴리텍 II 대학</t>
+          <t>한국폴리텍 III 대학</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -30309,7 +30313,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅱ대학남인천캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅲ대학강릉캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -30324,14 +30328,14 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅲ대학</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>한국폴리텍 II 대학</t>
+          <t>한국폴리텍 III 대학</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -30341,7 +30345,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅱ대학화성캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅲ대학원주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -30356,7 +30360,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅲ대학</t>
         </is>
       </c>
     </row>
@@ -30373,7 +30377,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅲ대학강릉캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅲ대학춘천캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -30388,14 +30392,14 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅲ대학</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>한국폴리텍 III 대학</t>
+          <t>한국폴리텍 IV 대학</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -30405,7 +30409,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅲ대학원주캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅳ대학아산캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -30420,14 +30424,14 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅳ대학</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>한국폴리텍 III 대학</t>
+          <t>한국폴리텍 IV 대학</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -30437,7 +30441,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅲ대학춘천캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅳ대학청주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -30452,7 +30456,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅳ대학</t>
         </is>
       </c>
     </row>
@@ -30469,7 +30473,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅳ대학아산캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅳ대학충남캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -30484,14 +30488,14 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅳ대학</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>한국폴리텍 IV 대학</t>
+          <t>한국폴리텍 V 대학</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -30501,7 +30505,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅳ대학청주캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅴ대학광주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -30516,14 +30520,14 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅴ대학</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>한국폴리텍 IV 대학</t>
+          <t>한국폴리텍 V 대학</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -30533,7 +30537,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅳ대학충남캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅴ대학순천캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -30548,7 +30552,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅴ대학</t>
         </is>
       </c>
     </row>
@@ -30565,7 +30569,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅴ대학광주캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅴ대학익산캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -30580,7 +30584,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅴ대학</t>
         </is>
       </c>
     </row>
@@ -30597,7 +30601,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅴ대학순천캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅴ대학전남캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -30612,7 +30616,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅴ대학</t>
         </is>
       </c>
     </row>
@@ -30629,7 +30633,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅴ대학익산캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅴ대학전북캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -30644,14 +30648,14 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅴ대학</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>한국폴리텍 V 대학</t>
+          <t>한국폴리텍 VI 대학</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -30661,7 +30665,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅴ대학전남캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅵ대학구미캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -30676,14 +30680,14 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅵ대학</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>한국폴리텍 V 대학</t>
+          <t>한국폴리텍 VI 대학</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -30693,7 +30697,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅴ대학전북캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅵ대학대구캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -30708,7 +30712,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅵ대학</t>
         </is>
       </c>
     </row>
@@ -30725,7 +30729,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅵ대학구미캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅵ대학영남융합기술캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -30740,7 +30744,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅵ대학</t>
         </is>
       </c>
     </row>
@@ -30757,7 +30761,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅵ대학대구캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅵ대학영주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -30772,14 +30776,14 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅵ대학</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>한국폴리텍 VI 대학</t>
+          <t>한국폴리텍 VII 대학</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -30789,7 +30793,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅵ대학영남융합기술캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅶ대학동부산캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -30804,14 +30808,14 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅶ대학</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>한국폴리텍 VI 대학</t>
+          <t>한국폴리텍 VII 대학</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -30821,7 +30825,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅵ대학영주캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅶ대학부산캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -30836,7 +30840,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅶ대학</t>
         </is>
       </c>
     </row>
@@ -30853,7 +30857,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅶ대학동부산캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅶ대학울산캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -30868,7 +30872,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅶ대학</t>
         </is>
       </c>
     </row>
@@ -30885,7 +30889,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅶ대학부산캠퍼스 도서관</t>
+          <t>한국폴리텍Ⅶ대학진주캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -30900,14 +30904,14 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍Ⅶ대학</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>한국폴리텍 VII 대학</t>
+          <t>한국폴리텍 특성화대학</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -30917,7 +30921,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅶ대학울산캠퍼스 도서관</t>
+          <t>한국폴리텍특성화 로봇캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -30932,14 +30936,14 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍특성화</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>한국폴리텍 VII 대학</t>
+          <t>한국폴리텍 특성화대학</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -30949,7 +30953,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>한국폴리텍Ⅶ대학진주캠퍼스 도서관</t>
+          <t>한국폴리텍특성화 바이오캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -30964,7 +30968,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍특성화</t>
         </is>
       </c>
     </row>
@@ -30981,7 +30985,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>한국폴리텍특성화 로봇캠퍼스 도서관</t>
+          <t>한국폴리텍특성화 반도체융합캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -30996,7 +31000,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>override</t>
+          <t>override:한국폴리텍특성화</t>
         </is>
       </c>
     </row>
@@ -31013,7 +31017,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>한국폴리텍특성화 바이오캠퍼스 도서관</t>
+          <t>한국폴리텍특성화 항공캠퍼스 도서관</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -31028,71 +31032,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>override</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>한국폴리텍 특성화대학</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>대학도서관</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>한국폴리텍특성화 반도체융합캠퍼스 도서관</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>KERIS</t>
-        </is>
-      </c>
-      <c r="E138" t="inlineStr">
-        <is>
-          <t>본교</t>
-        </is>
-      </c>
-      <c r="F138" t="inlineStr">
-        <is>
-          <t>override</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>한국폴리텍 특성화대학</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>대학도서관</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>한국폴리텍특성화 항공캠퍼스 도서관</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>KERIS</t>
-        </is>
-      </c>
-      <c r="E139" t="inlineStr">
-        <is>
-          <t>본교</t>
-        </is>
-      </c>
-      <c r="F139" t="inlineStr">
-        <is>
-          <t>override</t>
+          <t>override:한국폴리텍특성화</t>
         </is>
       </c>
     </row>

</xml_diff>